<commit_message>
@ Add optional delivery origin (출발지) to dispatch orders
Task C ①. Dispatch orders carry only a destination today; operators want
an optional origin so a delivery can start from a specified point instead
of always the bike position.

- DispatchOrder gains nullable originAddress / originLatitude /
  originLongitude (V40). Null = use bike current position (no extra logic).
- Dispatch Excel gains a "출발지 주소 (선택)" column: regular flow reads it
  at column index 4, sequential flow at index 5 (after 순번). Frontend
  geocodes the origin address alongside the destination; a failed origin
  geocode demotes the row to ERROR.
- DispatchBulkApplyRow / DispatchOrderCreateRequest / DispatchOrderReadResponse
  carry origin; appendForBike gains a 9-arg overload (6-arg delegates with
  nulls). export() emits the origin column.
- 차량 상세 배차 큐 row shows an 출발지 line when an origin is set.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/development/service-ops-api/src/main/resources/templates/excel/dispatch-template.xlsx
+++ b/development/service-ops-api/src/main/resources/templates/excel/dispatch-template.xlsx
@@ -498,13 +498,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D500"/>
+  <dimension ref="A1:E500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -535,6 +536,11 @@
           <t>배송지주소 *</t>
         </is>
       </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>출발지 주소 (선택)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -557,6 +563,11 @@
           <t>서울특별시 강남구 테헤란로 123</t>
         </is>
       </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 테헤란로 1</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -3574,7 +3585,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="B3:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">

</xml_diff>